<commit_message>
docs: deliver v3 effect workbook and cross-device review handoff
</commit_message>
<xml_diff>
--- a/outputs/01a151d0-9d92-7900-b5be-31a811469c9d/풀로세움_효과와스킬_분류_v2.xlsx
+++ b/outputs/01a151d0-9d92-7900-b5be-31a811469c9d/풀로세움_효과와스킬_분류_v2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soosa\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\soosa\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C67AAC0-B677-475F-B693-ADB5BD5E9CFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8F527C-0F85-4559-8C8E-6230DC4E6B42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="효과 분류" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="661" uniqueCount="468">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="473">
   <si>
     <t>풀로세움 효과 분류</t>
   </si>
@@ -85,9 +85,6 @@
     <t>공격력</t>
   </si>
   <si>
-    <t>분노</t>
-  </si>
-  <si>
     <t>공격력이 증가한다. 각 중첩의 남은 턴을 따로 센다.</t>
   </si>
   <si>
@@ -106,9 +103,6 @@
     <t>방어력</t>
   </si>
   <si>
-    <t>강인함</t>
-  </si>
-  <si>
     <t>방어력이 증가한다. 각 중첩의 남은 턴을 따로 센다.</t>
   </si>
   <si>
@@ -157,9 +151,6 @@
     <t>기존 약화의 명칭 제안</t>
   </si>
   <si>
-    <t>부식</t>
-  </si>
-  <si>
     <t>방어력이 감소한다. 각 중첩의 남은 턴을 따로 센다.</t>
   </si>
   <si>
@@ -196,9 +187,6 @@
     <t>가능</t>
   </si>
   <si>
-    <t>미정</t>
-  </si>
-  <si>
     <t>물 공격에 해제하는 기존 규칙</t>
   </si>
   <si>
@@ -211,9 +199,6 @@
     <t>겹 감소</t>
   </si>
   <si>
-    <t>기존 5겹과 자연 감소 기준은 재검토 전 기록</t>
-  </si>
-  <si>
     <t>출혈</t>
   </si>
   <si>
@@ -229,72 +214,33 @@
     <t>감전</t>
   </si>
   <si>
-    <t>지속 중 확률로 마비를 일으킨다. 마비의 행동 취소는 검토 대기다.</t>
-  </si>
-  <si>
-    <t>마비가 발동하면 감전을 소비하는 기존 안</t>
-  </si>
-  <si>
     <t>빙결</t>
   </si>
   <si>
     <t>겹이 쌓여 얼음으로 이어진다. 얼음의 행동 취소는 검토 대기다.</t>
   </si>
   <si>
-    <t>불 공격에 해제하는 기존 규칙</t>
-  </si>
-  <si>
-    <t>덩굴</t>
-  </si>
-  <si>
     <t>기술 하나의 사용을 제한한다.</t>
   </si>
   <si>
     <t>젖음</t>
   </si>
   <si>
-    <t>기동성·정확도·방어에 불리하며 전기·빙결과 연계한다.</t>
-  </si>
-  <si>
     <t>복합 상태 하나. 별도 수치 디버프로 중복 계산하지 않음</t>
   </si>
   <si>
     <t>교체 행동을 제한한다.</t>
   </si>
   <si>
-    <t>뿌리형은 불 공격에도 해제하는 기존 규칙</t>
-  </si>
-  <si>
     <t>도발</t>
   </si>
   <si>
-    <t>방어와 회피 행동을 제한한다.</t>
-  </si>
-  <si>
-    <t>반사를 함께 제한할지는 미정</t>
-  </si>
-  <si>
-    <t>봉인</t>
-  </si>
-  <si>
-    <t>지정된 기술의 사용을 제한한다.</t>
-  </si>
-  <si>
-    <t>덩굴과 통합 여부는 검토 중</t>
-  </si>
-  <si>
     <t>그늘</t>
   </si>
   <si>
-    <t>정해진 기간의 자연 햇빛 획득을 막는다.</t>
-  </si>
-  <si>
     <t>직접 전환·기존 보유 햇빛까지 없애지는 않음</t>
   </si>
   <si>
-    <t>숨막힘</t>
-  </si>
-  <si>
     <t>포자가 터진 뒤 해당 턴의 자연 햇빛 획득을 막는다.</t>
   </si>
   <si>
@@ -316,34 +262,13 @@
     <t>발동까지</t>
   </si>
   <si>
-    <t>발동 시 소모. 불 공격에 제거</t>
-  </si>
-  <si>
-    <t>기생 씨앗</t>
-  </si>
-  <si>
     <t>상대에게 지속 피해를 주고 연결된 쪽이 회복한다.</t>
   </si>
   <si>
-    <t>횟수</t>
-  </si>
-  <si>
     <t>상태 유지·턴 진행</t>
   </si>
   <si>
-    <t>교체 후 회복 대상·연결 판정은 검토 대기</t>
-  </si>
-  <si>
-    <t>타들어가는 갈망</t>
-  </si>
-  <si>
     <t>화상 조건을 만족하는 동안 자연 햇빛 획득을 막는다.</t>
-  </si>
-  <si>
-    <t>교체 후 대면·화상 조건 판정은 검토 대기</t>
-  </si>
-  <si>
-    <t>지옥의 불씨</t>
   </si>
   <si>
     <t>기존 화상이 있으면 화상 추가 피해를 준다. 첫 불 공격은 공격 스킬이다.</t>
@@ -1425,11 +1350,126 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>치명</t>
+    <t>속박</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>속박</t>
+    <t>고정 없음</t>
+  </si>
+  <si>
+    <t>최대 5겹. 2턴 동안 재부여가 없으면 매 턴 1겹씩 감소</t>
+  </si>
+  <si>
+    <t>약한 피해를 주며, 지속 중 확률로 마비를 일으킨다. 마비의 행동 취소는 검토 대기다.</t>
+  </si>
+  <si>
+    <t>2턴 동안 재부여가 없으면 매 턴 1겹씩 감소. 불 공격에도 해제</t>
+  </si>
+  <si>
+    <t>이번 턴</t>
+  </si>
+  <si>
+    <t>억셈</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>시듦</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>활력</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>예리</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>마비 발동 시 소비하는 기존 안</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>봉인</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>기동성·정확도·방어에 불리하며 전기·빙결과 연계한다.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>힌식물에게 여러 번 사용 금지. 교체 되면 초기화. 1:1에서는 봉인같은 걸로 취급할지 논의</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>방어스킬을 전부 제한한다.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>방어스킬+다른스킬에 관해서는 어떻게 할 지 논의</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>기존 봉인은 폐기</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>정해진 기간의 자연 햇빛 획득을 막는다. 얘는 환경스킬로 옮기자.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>암실</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>기생</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>기간</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>다음 턴부터 턴 끝마다 1겹 증가. 3겹 도달 시 발동·소모. 불 공격에 제거</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>교체 후 회복 대상·연결 판정은 검토 대기. 원래는 횟수였는데 이게 기간이랑 다른게 뭔지 봐줘</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>얘도 새로운 상태이상이 아닌 화상의 중첩느낌으로 하자. 화상은 독처럼 중첩이 없었으나 이 스킬이 붙으면 중첩이 되는 ui로 바꾸는 걸로. 새로운 상태이상으로 취급하지는 말자.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>가능</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>화상이 해제 되면 자연스레 해제</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>상대의 이로운 효과 제거에는 적용</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>사용시 해제</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>내가 다음타 공격하거나, 빗나감 실패시</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>지옥 불</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>갈증</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>얘는 새로운 상태이상으로 만들지 말고 화상+암실 계속 갱신이 좋을 듯. 이름은 갈증으로</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -1635,7 +1675,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1721,45 +1761,93 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1772,9 +1860,6 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -1785,54 +1870,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2052,12 +2089,12 @@
     <tabColor rgb="FF244B61"/>
   </sheetPr>
   <dimension ref="A1:J52"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="4" max="4" width="15.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
     <col min="7" max="7" width="13" customWidth="1"/>
@@ -2066,7 +2103,7 @@
     <col min="10" max="10" width="37" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5">
+    <row r="1" spans="1:10" ht="17">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2079,20 +2116,20 @@
       <c r="J1" s="1"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
-      <c r="A2" s="29" t="s">
+      <c r="A2" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-      <c r="J2" s="29"/>
-    </row>
-    <row r="3" spans="1:10" ht="16.5">
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+    </row>
+    <row r="3" spans="1:10" ht="17">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -2104,55 +2141,55 @@
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
     </row>
-    <row r="4" spans="1:10" ht="23.1" customHeight="1">
-      <c r="A4" s="30" t="s">
+    <row r="4" spans="1:10" ht="23.15" customHeight="1">
+      <c r="A4" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="31" t="s">
+      <c r="B4" s="53"/>
+      <c r="C4" s="53"/>
+      <c r="D4" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
-    </row>
-    <row r="5" spans="1:10" ht="23.1" customHeight="1">
-      <c r="A5" s="30" t="s">
+      <c r="E4" s="54"/>
+      <c r="F4" s="54"/>
+      <c r="G4" s="54"/>
+      <c r="H4" s="54"/>
+      <c r="I4" s="54"/>
+      <c r="J4" s="54"/>
+    </row>
+    <row r="5" spans="1:10" ht="23.15" customHeight="1">
+      <c r="A5" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="30"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="31" t="s">
+      <c r="B5" s="53"/>
+      <c r="C5" s="53"/>
+      <c r="D5" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
-    </row>
-    <row r="6" spans="1:10" ht="23.1" customHeight="1">
-      <c r="A6" s="30" t="s">
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+    </row>
+    <row r="6" spans="1:10" ht="23.15" customHeight="1">
+      <c r="A6" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="30"/>
-      <c r="C6" s="30"/>
-      <c r="D6" s="31" t="s">
+      <c r="B6" s="53"/>
+      <c r="C6" s="53"/>
+      <c r="D6" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="31"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="31"/>
-    </row>
-    <row r="7" spans="1:10" ht="16.5">
+      <c r="E6" s="54"/>
+      <c r="F6" s="54"/>
+      <c r="G6" s="54"/>
+      <c r="H6" s="54"/>
+      <c r="I6" s="54"/>
+      <c r="J6" s="54"/>
+    </row>
+    <row r="7" spans="1:10" ht="17">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -2197,1239 +2234,1219 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="42" customHeight="1">
-      <c r="A9" s="32" t="s">
+      <c r="A9" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="46" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>19</v>
       </c>
       <c r="D9" s="26" t="s">
+        <v>449</v>
+      </c>
+      <c r="E9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="22" t="s">
+      <c r="G9" s="22" t="s">
         <v>22</v>
-      </c>
-      <c r="G9" s="22" t="s">
-        <v>23</v>
       </c>
       <c r="H9" s="23">
         <v>5</v>
       </c>
       <c r="I9" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="9" t="s">
+    </row>
+    <row r="10" spans="1:10" ht="42" customHeight="1">
+      <c r="A10" s="47"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="7" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="42" customHeight="1">
-      <c r="A10" s="33"/>
-      <c r="B10" s="33"/>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="3" t="s">
+        <v>447</v>
+      </c>
+      <c r="E10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>28</v>
-      </c>
       <c r="F10" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G10" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G10" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H10" s="25">
         <v>5</v>
       </c>
       <c r="I10" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="J10" s="1" t="s">
-        <v>25</v>
-      </c>
     </row>
     <row r="11" spans="1:10" ht="42" customHeight="1">
-      <c r="A11" s="33"/>
-      <c r="B11" s="33"/>
+      <c r="A11" s="47"/>
+      <c r="B11" s="47"/>
       <c r="C11" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>31</v>
-      </c>
       <c r="F11" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H11" s="25">
         <v>5</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J11" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="42" customHeight="1">
+      <c r="A12" s="47"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>450</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="42" customHeight="1">
-      <c r="A12" s="33"/>
-      <c r="B12" s="33"/>
-      <c r="C12" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>466</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="F12" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G12" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H12" s="25">
         <v>5</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J12" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="42" customHeight="1">
+      <c r="A13" s="47"/>
+      <c r="B13" s="47"/>
+      <c r="C13" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>439</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="42" customHeight="1">
-      <c r="A13" s="33"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>464</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>37</v>
-      </c>
       <c r="F13" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G13" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H13" s="25">
         <v>5</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="42" customHeight="1">
-      <c r="A14" s="34" t="s">
-        <v>38</v>
-      </c>
-      <c r="B14" s="34" t="s">
-        <v>39</v>
+      <c r="A14" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="48" t="s">
+        <v>37</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>19</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="F14" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="22" t="s">
         <v>22</v>
-      </c>
-      <c r="G14" s="22" t="s">
-        <v>23</v>
       </c>
       <c r="H14" s="23">
         <v>5</v>
       </c>
       <c r="I14" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="42" customHeight="1">
-      <c r="A15" s="35"/>
-      <c r="B15" s="35"/>
+      <c r="A15" s="49"/>
+      <c r="B15" s="49"/>
       <c r="C15" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>44</v>
+        <v>448</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F15" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G15" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H15" s="25">
         <v>5</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="42" customHeight="1">
-      <c r="A16" s="35"/>
-      <c r="B16" s="35"/>
+      <c r="A16" s="49"/>
+      <c r="B16" s="49"/>
       <c r="C16" s="10" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F16" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G16" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H16" s="25">
         <v>5</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="33.950000000000003" customHeight="1">
-      <c r="A17" s="35"/>
-      <c r="B17" s="35"/>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" ht="34" customHeight="1">
+      <c r="A17" s="49"/>
+      <c r="B17" s="49"/>
       <c r="C17" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F17" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G17" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H17" s="25">
         <v>5</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="42" customHeight="1">
-      <c r="A18" s="35"/>
-      <c r="B18" s="35"/>
+      <c r="A18" s="49"/>
+      <c r="B18" s="49"/>
       <c r="C18" s="10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>465</v>
+        <v>440</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F18" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G18" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H18" s="25">
         <v>5</v>
       </c>
       <c r="I18" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J18" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="42" customHeight="1">
+      <c r="A19" s="50"/>
+      <c r="B19" s="50" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="50" t="s">
+        <v>50</v>
+      </c>
+      <c r="D19" s="26" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="1:10" ht="42" customHeight="1">
-      <c r="A19" s="36"/>
-      <c r="B19" s="36" t="s">
+      <c r="E19" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="36" t="s">
+      <c r="F19" s="22" t="s">
         <v>53</v>
       </c>
-      <c r="D19" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="F19" s="22" t="s">
-        <v>56</v>
-      </c>
       <c r="G19" s="22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H19" s="23">
         <v>3</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J19" s="9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="42" customHeight="1">
+      <c r="A20" s="51"/>
+      <c r="B20" s="51"/>
+      <c r="C20" s="51"/>
+      <c r="D20" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="F20" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="H20" s="25" t="s">
+        <v>442</v>
+      </c>
+      <c r="I20" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="J20" s="1" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="42" customHeight="1">
+      <c r="A21" s="51"/>
+      <c r="B21" s="51"/>
+      <c r="C21" s="55"/>
+      <c r="D21" s="62" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="20" spans="1:10" ht="42" customHeight="1">
-      <c r="A20" s="46"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="46"/>
-      <c r="D20" s="47" t="s">
+      <c r="E21" s="63" t="s">
         <v>59</v>
       </c>
-      <c r="E20" s="48" t="s">
+      <c r="F21" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G21" s="64" t="s">
+        <v>22</v>
+      </c>
+      <c r="H21" s="65">
+        <v>3</v>
+      </c>
+      <c r="I21" s="64" t="s">
+        <v>23</v>
+      </c>
+      <c r="J21" s="63" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="G20" s="49" t="s">
+    </row>
+    <row r="22" spans="1:10" ht="42" customHeight="1">
+      <c r="A22" s="51"/>
+      <c r="B22" s="51"/>
+      <c r="C22" s="56"/>
+      <c r="D22" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="E22" s="30" t="s">
+        <v>444</v>
+      </c>
+      <c r="F22" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H22" s="32">
+        <v>3</v>
+      </c>
+      <c r="I22" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="30" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="42" customHeight="1">
+      <c r="A23" s="51"/>
+      <c r="B23" s="51"/>
+      <c r="C23" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="H20" s="50" t="inlineStr">
-        <is>
-          <t>고정 없음</t>
-        </is>
-      </c>
-      <c r="I20" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J20" s="48" t="inlineStr">
-        <is>
-          <t>최대 5겹. 2턴 동안 재부여가 없으면 매 턴 1겹씩 감소</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="42" customHeight="1">
-      <c r="A21" s="46"/>
-      <c r="B21" s="46"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="52" t="s">
+      <c r="D23" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="53" t="s">
+      <c r="E23" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="F21" s="54" t="s">
-        <v>42</v>
-      </c>
-      <c r="G21" s="54" t="s">
+      <c r="F23" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G23" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="H23" s="25" t="s">
+        <v>442</v>
+      </c>
+      <c r="I23" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="H21" s="55">
+      <c r="J23" s="1" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="42" customHeight="1">
+      <c r="A24" s="51"/>
+      <c r="B24" s="51"/>
+      <c r="C24" s="51"/>
+      <c r="D24" s="3" t="s">
+        <v>452</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F24" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G24" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="25">
+        <v>1</v>
+      </c>
+      <c r="I24" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="1:10" ht="42" customHeight="1">
+      <c r="A25" s="51"/>
+      <c r="B25" s="51"/>
+      <c r="C25" s="51"/>
+      <c r="D25" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>453</v>
+      </c>
+      <c r="F25" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="25">
         <v>3</v>
       </c>
-      <c r="I21" s="54" t="s">
-        <v>24</v>
-      </c>
-      <c r="J21" s="53" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="42" customHeight="1">
-      <c r="A22" s="46"/>
-      <c r="B22" s="46"/>
-      <c r="C22" s="56"/>
-      <c r="D22" s="57" t="s">
+      <c r="I25" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="J25" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="58" t="inlineStr">
-        <is>
-          <t>약한 피해를 주며, 지속 중 확률로 마비를 일으킨다. 마비의 행동 취소는 검토 대기다.</t>
-        </is>
-      </c>
-      <c r="F22" s="59" t="s">
-        <v>56</v>
-      </c>
-      <c r="G22" s="59" t="s">
+    </row>
+    <row r="26" spans="1:10" ht="42" customHeight="1">
+      <c r="A26" s="51"/>
+      <c r="B26" s="51"/>
+      <c r="C26" s="51"/>
+      <c r="D26" s="3" t="s">
+        <v>441</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="F26" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G26" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="25">
+        <v>3</v>
+      </c>
+      <c r="I26" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="H22" s="60">
+      <c r="J26" s="1" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="42" customHeight="1">
+      <c r="A27" s="51"/>
+      <c r="B27" s="51"/>
+      <c r="C27" s="51"/>
+      <c r="D27" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>455</v>
+      </c>
+      <c r="F27" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G27" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="25">
+        <v>1</v>
+      </c>
+      <c r="I27" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="42" customHeight="1">
+      <c r="A28" s="51"/>
+      <c r="B28" s="51"/>
+      <c r="C28" s="51"/>
+      <c r="D28" s="3" t="s">
+        <v>457</v>
+      </c>
+      <c r="E28" s="1"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="1"/>
+    </row>
+    <row r="29" spans="1:10" ht="42" customHeight="1">
+      <c r="A29" s="51"/>
+      <c r="B29" s="51"/>
+      <c r="C29" s="51"/>
+      <c r="D29" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="F29" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="25" t="s">
+        <v>446</v>
+      </c>
+      <c r="I29" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="J29" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="42" customHeight="1">
+      <c r="A30" s="51"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="55"/>
+      <c r="D30" s="29" t="s">
+        <v>459</v>
+      </c>
+      <c r="E30" s="30" t="s">
+        <v>72</v>
+      </c>
+      <c r="F30" s="31" t="s">
+        <v>465</v>
+      </c>
+      <c r="G30" s="31" t="s">
+        <v>73</v>
+      </c>
+      <c r="H30" s="32"/>
+      <c r="I30" s="31" t="s">
+        <v>23</v>
+      </c>
+      <c r="J30" s="30" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="42" customHeight="1">
+      <c r="A31" s="51"/>
+      <c r="B31" s="51"/>
+      <c r="C31" s="56" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" s="33" t="s">
+        <v>76</v>
+      </c>
+      <c r="E31" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="F31" s="35" t="s">
+        <v>53</v>
+      </c>
+      <c r="G31" s="35" t="s">
+        <v>78</v>
+      </c>
+      <c r="H31" s="36" t="s">
+        <v>442</v>
+      </c>
+      <c r="I31" s="35" t="s">
+        <v>23</v>
+      </c>
+      <c r="J31" s="34" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="42" customHeight="1">
+      <c r="A32" s="51"/>
+      <c r="B32" s="51"/>
+      <c r="C32" s="51"/>
+      <c r="D32" s="3" t="s">
+        <v>460</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F32" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G32" s="24" t="s">
+        <v>461</v>
+      </c>
+      <c r="H32" s="25">
+        <v>3</v>
+      </c>
+      <c r="I32" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="42" customHeight="1">
+      <c r="A33" s="51"/>
+      <c r="B33" s="51"/>
+      <c r="C33" s="51"/>
+      <c r="D33" s="3" t="s">
+        <v>471</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F33" s="24" t="s">
+        <v>466</v>
+      </c>
+      <c r="G33" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="H33" s="25">
         <v>2</v>
       </c>
-      <c r="I22" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="J22" s="58" t="inlineStr">
-        <is>
-          <t>걸린 턴 + 이후 2턴. 마비 발동 시 소비하는 기존 안</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="42" customHeight="1">
-      <c r="A23" s="46"/>
-      <c r="B23" s="46"/>
-      <c r="C23" s="56" t="inlineStr">
-        <is>
-          <t>비데미지</t>
-        </is>
-      </c>
-      <c r="D23" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="E23" s="48" t="s">
-        <v>71</v>
-      </c>
-      <c r="F23" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="G23" s="49" t="s">
-        <v>61</v>
-      </c>
-      <c r="H23" s="50" t="inlineStr">
-        <is>
-          <t>고정 없음</t>
-        </is>
-      </c>
-      <c r="I23" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J23" s="48" t="inlineStr">
-        <is>
-          <t>2턴 동안 재부여가 없으면 매 턴 1겹씩 감소. 불 공격에도 해제</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="42" customHeight="1">
-      <c r="A24" s="46"/>
-      <c r="B24" s="46"/>
-      <c r="C24" s="46"/>
-      <c r="D24" s="47" t="s">
-        <v>73</v>
-      </c>
-      <c r="E24" s="48" t="s">
-        <v>74</v>
-      </c>
-      <c r="F24" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="G24" s="49" t="s">
+      <c r="I33" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="J33" s="1" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="42" customHeight="1">
+      <c r="A34" s="51"/>
+      <c r="B34" s="51"/>
+      <c r="C34" s="55"/>
+      <c r="D34" s="29" t="s">
+        <v>470</v>
+      </c>
+      <c r="E34" s="30" t="s">
+        <v>82</v>
+      </c>
+      <c r="F34" s="31" t="s">
+        <v>466</v>
+      </c>
+      <c r="G34" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="H34" s="32">
+        <v>2</v>
+      </c>
+      <c r="I34" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="J34" s="30" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="42" customHeight="1">
+      <c r="A35" s="51"/>
+      <c r="B35" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="C35" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="D35" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="E35" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="F35" s="40" t="s">
+        <v>467</v>
+      </c>
+      <c r="G35" s="40" t="s">
+        <v>461</v>
+      </c>
+      <c r="H35" s="41">
+        <v>3</v>
+      </c>
+      <c r="I35" s="40" t="s">
         <v>23</v>
       </c>
-      <c r="H24" s="50">
-        <v>1</v>
-      </c>
-      <c r="I24" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J24" s="48" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="42" customHeight="1">
-      <c r="A25" s="46"/>
-      <c r="B25" s="46"/>
-      <c r="C25" s="46"/>
-      <c r="D25" s="47" t="s">
-        <v>75</v>
-      </c>
-      <c r="E25" s="48" t="s">
-        <v>76</v>
-      </c>
-      <c r="F25" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="G25" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="H25" s="50">
-        <v>2</v>
-      </c>
-      <c r="I25" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J25" s="48" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="42" customHeight="1">
-      <c r="A26" s="46"/>
-      <c r="B26" s="46"/>
-      <c r="C26" s="46"/>
-      <c r="D26" s="47" t="s">
-        <v>467</v>
-      </c>
-      <c r="E26" s="48" t="s">
-        <v>78</v>
-      </c>
-      <c r="F26" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="G26" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="H26" s="50">
-        <v>2</v>
-      </c>
-      <c r="I26" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J26" s="48" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="42" customHeight="1">
-      <c r="A27" s="46"/>
-      <c r="B27" s="46"/>
-      <c r="C27" s="46"/>
-      <c r="D27" s="47" t="s">
-        <v>80</v>
-      </c>
-      <c r="E27" s="48" t="s">
-        <v>81</v>
-      </c>
-      <c r="F27" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="G27" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="H27" s="50">
-        <v>1</v>
-      </c>
-      <c r="I27" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J27" s="48" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="42" customHeight="1">
-      <c r="A28" s="46"/>
-      <c r="B28" s="46"/>
-      <c r="C28" s="46"/>
-      <c r="D28" s="47" t="s">
-        <v>83</v>
-      </c>
-      <c r="E28" s="48" t="s">
-        <v>84</v>
-      </c>
-      <c r="F28" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="G28" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="H28" s="50">
-        <v>2</v>
-      </c>
-      <c r="I28" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J28" s="48" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="42" customHeight="1">
-      <c r="A29" s="46"/>
-      <c r="B29" s="46"/>
-      <c r="C29" s="46"/>
-      <c r="D29" s="47" t="s">
-        <v>86</v>
-      </c>
-      <c r="E29" s="48" t="s">
+      <c r="J35" s="39" t="s">
         <v>87</v>
       </c>
-      <c r="F29" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="G29" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="H29" s="50" t="inlineStr">
-        <is>
-          <t>이번 턴</t>
-        </is>
-      </c>
-      <c r="I29" s="49" t="s">
-        <v>24</v>
-      </c>
-      <c r="J29" s="48" t="s">
+    </row>
+    <row r="36" spans="1:10" ht="42" customHeight="1">
+      <c r="A36" s="51"/>
+      <c r="B36" s="51"/>
+      <c r="C36" s="56" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" ht="42" customHeight="1">
-      <c r="A30" s="46"/>
-      <c r="B30" s="46"/>
-      <c r="C30" s="51"/>
-      <c r="D30" s="52" t="s">
+      <c r="D36" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E30" s="53" t="s">
+      <c r="E36" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F30" s="54" t="s">
-        <v>42</v>
-      </c>
-      <c r="G30" s="54" t="s">
-        <v>91</v>
-      </c>
-      <c r="H30" s="55"/>
-      <c r="I30" s="54" t="s">
-        <v>24</v>
-      </c>
-      <c r="J30" s="53" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="42" customHeight="1">
-      <c r="A31" s="46"/>
-      <c r="B31" s="46"/>
-      <c r="C31" s="56" t="s">
-        <v>93</v>
-      </c>
-      <c r="D31" s="57" t="s">
-        <v>94</v>
-      </c>
-      <c r="E31" s="58" t="s">
-        <v>95</v>
-      </c>
-      <c r="F31" s="59" t="s">
-        <v>56</v>
-      </c>
-      <c r="G31" s="59" t="s">
-        <v>96</v>
-      </c>
-      <c r="H31" s="60" t="inlineStr">
-        <is>
-          <t>고정 없음</t>
-        </is>
-      </c>
-      <c r="I31" s="59" t="s">
-        <v>24</v>
-      </c>
-      <c r="J31" s="58" t="inlineStr">
-        <is>
-          <t>다음 턴부터 턴 끝마다 1겹 증가. 3겹 도달 시 발동·소모. 불 공격에 제거</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="42" customHeight="1">
-      <c r="A32" s="46"/>
-      <c r="B32" s="46"/>
-      <c r="C32" s="46"/>
-      <c r="D32" s="47" t="s">
-        <v>98</v>
-      </c>
-      <c r="E32" s="48" t="s">
-        <v>99</v>
-      </c>
-      <c r="F32" s="49" t="s">
-        <v>56</v>
-      </c>
-      <c r="G32" s="49" t="s">
-        <v>100</v>
-      </c>
-      <c r="H32" s="50">
-        <v>3</v>
-      </c>
-      <c r="I32" s="49" t="s">
-        <v>101</v>
-      </c>
-      <c r="J32" s="48" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="42" customHeight="1">
-      <c r="A33" s="46"/>
-      <c r="B33" s="46"/>
-      <c r="C33" s="46"/>
-      <c r="D33" s="47" t="s">
-        <v>103</v>
-      </c>
-      <c r="E33" s="48" t="s">
-        <v>104</v>
-      </c>
-      <c r="F33" s="49" t="s">
-        <v>42</v>
-      </c>
-      <c r="G33" s="49" t="s">
-        <v>23</v>
-      </c>
-      <c r="H33" s="50">
-        <v>2</v>
-      </c>
-      <c r="I33" s="49" t="s">
-        <v>101</v>
-      </c>
-      <c r="J33" s="48" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="42" customHeight="1">
-      <c r="A34" s="46"/>
-      <c r="B34" s="46"/>
-      <c r="C34" s="51"/>
-      <c r="D34" s="52" t="s">
-        <v>106</v>
-      </c>
-      <c r="E34" s="53" t="s">
-        <v>107</v>
-      </c>
-      <c r="F34" s="54" t="s">
-        <v>42</v>
-      </c>
-      <c r="G34" s="54" t="s">
-        <v>23</v>
-      </c>
-      <c r="H34" s="55">
-        <v>2</v>
-      </c>
-      <c r="I34" s="54" t="s">
-        <v>101</v>
-      </c>
-      <c r="J34" s="53" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="42" customHeight="1">
-      <c r="A35" s="46"/>
-      <c r="B35" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="C35" s="61" t="s">
-        <v>109</v>
-      </c>
-      <c r="D35" s="62" t="s">
-        <v>110</v>
-      </c>
-      <c r="E35" s="63" t="s">
-        <v>111</v>
-      </c>
-      <c r="F35" s="64" t="s">
+      <c r="F36" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G36" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G35" s="64" t="s">
-        <v>100</v>
-      </c>
-      <c r="H35" s="65">
-        <v>3</v>
-      </c>
-      <c r="I35" s="64" t="s">
-        <v>24</v>
-      </c>
-      <c r="J35" s="63" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="42" customHeight="1">
-      <c r="A36" s="46"/>
-      <c r="B36" s="37"/>
-      <c r="C36" s="56" t="s">
-        <v>113</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="F36" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="G36" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H36" s="25">
         <v>1</v>
       </c>
       <c r="I36" s="24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>116</v>
+        <v>91</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="42" customHeight="1">
-      <c r="A37" s="66"/>
-      <c r="B37" s="66"/>
-      <c r="C37" s="66"/>
+      <c r="A37" s="52"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="52"/>
       <c r="D37" s="3" t="s">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="F37" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="G37" s="24" t="s">
+      <c r="H37" s="25">
+        <v>3</v>
+      </c>
+      <c r="I37" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="H37" s="25" t="s">
-        <v>57</v>
-      </c>
-      <c r="I37" s="24" t="s">
-        <v>24</v>
-      </c>
       <c r="J37" s="1" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="42" customHeight="1">
-      <c r="A38" s="38" t="s">
+      <c r="A38" s="43" t="s">
         <v>5</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>121</v>
+        <v>96</v>
       </c>
       <c r="D38" s="26" t="s">
-        <v>122</v>
+        <v>97</v>
       </c>
       <c r="E38" s="9" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="F38" s="22" t="s">
-        <v>22</v>
+        <v>467</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>124</v>
+        <v>468</v>
       </c>
       <c r="H38" s="23"/>
       <c r="I38" s="22" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J38" s="9" t="s">
-        <v>126</v>
+        <v>101</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="42" customHeight="1">
-      <c r="A39" s="39"/>
+      <c r="A39" s="44"/>
       <c r="B39" s="14" t="s">
-        <v>127</v>
+        <v>102</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>129</v>
+        <v>104</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="F39" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="G39" s="24" t="s">
-        <v>124</v>
+        <v>105</v>
+      </c>
+      <c r="F39" s="22" t="s">
+        <v>467</v>
+      </c>
+      <c r="G39" s="22" t="s">
+        <v>469</v>
       </c>
       <c r="H39" s="25"/>
       <c r="I39" s="24" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>131</v>
+        <v>106</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="42" customHeight="1">
-      <c r="A40" s="39"/>
+      <c r="A40" s="44"/>
       <c r="B40" s="14" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>134</v>
+        <v>109</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F40" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="G40" s="24" t="s">
-        <v>124</v>
+        <v>110</v>
+      </c>
+      <c r="F40" s="22" t="s">
+        <v>467</v>
+      </c>
+      <c r="G40" s="22" t="s">
+        <v>468</v>
       </c>
       <c r="H40" s="25"/>
       <c r="I40" s="24" t="s">
-        <v>125</v>
+        <v>100</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="42" customHeight="1">
-      <c r="A41" s="40" t="s">
-        <v>137</v>
-      </c>
-      <c r="B41" s="40" t="s">
-        <v>138</v>
+      <c r="A41" s="45" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="45" t="s">
+        <v>113</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>139</v>
+        <v>114</v>
       </c>
       <c r="D41" s="26" t="s">
-        <v>140</v>
+        <v>115</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>141</v>
+        <v>116</v>
       </c>
       <c r="F41" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="22" t="s">
         <v>22</v>
-      </c>
-      <c r="G41" s="22" t="s">
-        <v>23</v>
       </c>
       <c r="H41" s="23">
         <v>2</v>
       </c>
       <c r="I41" s="22" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="J41" s="9" t="s">
-        <v>143</v>
+        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="42" customHeight="1">
-      <c r="A42" s="41"/>
-      <c r="B42" s="41"/>
+      <c r="A42" s="42"/>
+      <c r="B42" s="42"/>
       <c r="C42" s="16" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>145</v>
+        <v>120</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>146</v>
+        <v>121</v>
       </c>
       <c r="F42" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G42" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H42" s="25">
         <v>3</v>
       </c>
       <c r="I42" s="24" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="J42" s="1" t="s">
-        <v>147</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="42" customHeight="1">
-      <c r="A43" s="41"/>
-      <c r="B43" s="41"/>
-      <c r="C43" s="41" t="s">
-        <v>148</v>
+      <c r="A43" s="42"/>
+      <c r="B43" s="42"/>
+      <c r="C43" s="42" t="s">
+        <v>123</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>150</v>
+        <v>125</v>
       </c>
       <c r="F43" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G43" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G43" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H43" s="25">
         <v>3</v>
       </c>
       <c r="I43" s="24" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="J43" s="1" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="42" customHeight="1">
-      <c r="A44" s="41"/>
-      <c r="B44" s="41"/>
-      <c r="C44" s="41"/>
+      <c r="A44" s="42"/>
+      <c r="B44" s="42"/>
+      <c r="C44" s="42"/>
       <c r="D44" s="3" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="F44" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G44" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G44" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H44" s="25">
         <v>3</v>
       </c>
       <c r="I44" s="24" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>151</v>
+        <v>126</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="42" customHeight="1">
-      <c r="A45" s="41"/>
-      <c r="B45" s="41"/>
-      <c r="C45" s="41"/>
+      <c r="A45" s="42"/>
+      <c r="B45" s="42"/>
+      <c r="C45" s="42"/>
       <c r="D45" s="3" t="s">
-        <v>154</v>
+        <v>129</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="F45" s="24" t="s">
+        <v>21</v>
+      </c>
+      <c r="G45" s="24" t="s">
         <v>22</v>
-      </c>
-      <c r="G45" s="24" t="s">
-        <v>23</v>
       </c>
       <c r="H45" s="25">
         <v>3</v>
       </c>
       <c r="I45" s="24" t="s">
-        <v>142</v>
+        <v>117</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="33.950000000000003" customHeight="1">
-      <c r="A46" s="41"/>
-      <c r="B46" s="41" t="s">
-        <v>156</v>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="34" customHeight="1">
+      <c r="A46" s="42"/>
+      <c r="B46" s="42" t="s">
+        <v>131</v>
       </c>
       <c r="C46" s="16" t="s">
-        <v>157</v>
+        <v>132</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>159</v>
+        <v>134</v>
       </c>
       <c r="F46" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G46" s="24" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H46" s="25"/>
       <c r="I46" s="24" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>161</v>
+        <v>136</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="42" customHeight="1">
-      <c r="A47" s="41"/>
-      <c r="B47" s="41"/>
+      <c r="A47" s="42"/>
+      <c r="B47" s="42"/>
       <c r="C47" s="16" t="s">
-        <v>162</v>
+        <v>137</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>163</v>
+        <v>138</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>164</v>
+        <v>139</v>
       </c>
       <c r="F47" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G47" s="24" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H47" s="25"/>
       <c r="I47" s="24" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="J47" s="1" t="s">
-        <v>165</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="42" customHeight="1">
-      <c r="A48" s="41"/>
-      <c r="B48" s="41"/>
+      <c r="A48" s="42"/>
+      <c r="B48" s="42"/>
       <c r="C48" s="16" t="s">
-        <v>166</v>
+        <v>141</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>168</v>
+        <v>143</v>
       </c>
       <c r="F48" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G48" s="24" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H48" s="25"/>
       <c r="I48" s="24" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="J48" s="1" t="s">
-        <v>169</v>
+        <v>144</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="42" customHeight="1">
-      <c r="A49" s="41"/>
-      <c r="B49" s="41"/>
+      <c r="A49" s="42"/>
+      <c r="B49" s="42"/>
       <c r="C49" s="16" t="s">
-        <v>144</v>
+        <v>119</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>171</v>
+        <v>146</v>
       </c>
       <c r="F49" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G49" s="24" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H49" s="25"/>
       <c r="I49" s="24" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="J49" s="1" t="s">
-        <v>172</v>
+        <v>147</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="42" customHeight="1">
-      <c r="A50" s="41"/>
-      <c r="B50" s="41"/>
+      <c r="A50" s="42"/>
+      <c r="B50" s="42"/>
       <c r="C50" s="16" t="s">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>174</v>
+        <v>149</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>175</v>
+        <v>150</v>
       </c>
       <c r="F50" s="24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G50" s="24" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H50" s="25"/>
       <c r="I50" s="24" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="J50" s="1" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="42" customHeight="1">
       <c r="A51" s="19" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>178</v>
+        <v>153</v>
       </c>
       <c r="C51" s="19" t="s">
-        <v>179</v>
+        <v>154</v>
       </c>
       <c r="D51" s="26" t="s">
-        <v>180</v>
+        <v>155</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>181</v>
+        <v>156</v>
       </c>
       <c r="F51" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H51" s="23"/>
       <c r="I51" s="22" t="s">
-        <v>182</v>
+        <v>157</v>
       </c>
       <c r="J51" s="9" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="57.95" customHeight="1">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="58" customHeight="1">
       <c r="A52" s="21" t="s">
-        <v>184</v>
+        <v>159</v>
       </c>
       <c r="B52" s="21" t="s">
-        <v>185</v>
+        <v>160</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>186</v>
+        <v>161</v>
       </c>
       <c r="D52" s="26" t="s">
-        <v>187</v>
+        <v>162</v>
       </c>
       <c r="E52" s="9" t="s">
-        <v>188</v>
+        <v>163</v>
       </c>
       <c r="F52" s="22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H52" s="23"/>
       <c r="I52" s="22" t="s">
-        <v>160</v>
+        <v>135</v>
       </c>
       <c r="J52" s="9" t="s">
-        <v>189</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A2:J2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="D4:J4"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="D5:J5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="D6:J6"/>
+    <mergeCell ref="A9:A13"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="A19:A37"/>
+    <mergeCell ref="C19:C22"/>
+    <mergeCell ref="C23:C30"/>
+    <mergeCell ref="C31:C34"/>
+    <mergeCell ref="C36:C37"/>
     <mergeCell ref="C43:C45"/>
     <mergeCell ref="A38:A40"/>
     <mergeCell ref="A41:A50"/>
@@ -3439,20 +3456,6 @@
     <mergeCell ref="B35:B37"/>
     <mergeCell ref="B41:B45"/>
     <mergeCell ref="B46:B50"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="D6:J6"/>
-    <mergeCell ref="A9:A13"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="A19:A37"/>
-    <mergeCell ref="C19:C22"/>
-    <mergeCell ref="C23:C30"/>
-    <mergeCell ref="C31:C34"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="D4:J4"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="D5:J5"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3465,7 +3468,7 @@
     <tabColor rgb="FF4D7188"/>
   </sheetPr>
   <dimension ref="A1:H26"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="17" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -3477,7 +3480,7 @@
     <col min="8" max="8" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.5">
+    <row r="1" spans="1:8" ht="17">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3488,18 +3491,18 @@
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="29" t="s">
-        <v>190</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-    </row>
-    <row r="3" spans="1:8" ht="16.5">
+      <c r="A2" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+    </row>
+    <row r="3" spans="1:8" ht="17">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -3509,7 +3512,7 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" ht="16.5">
+    <row r="4" spans="1:8" ht="17">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -3521,554 +3524,554 @@
     </row>
     <row r="5" spans="1:8" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>191</v>
+        <v>166</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>192</v>
+        <v>167</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>193</v>
+        <v>168</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="42" customHeight="1">
+      <c r="A6" s="46" t="s">
+        <v>173</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="42" customHeight="1">
+      <c r="A7" s="47"/>
+      <c r="B7" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>182</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="34" customHeight="1">
+      <c r="A8" s="48" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>188</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="34" customHeight="1">
+      <c r="A9" s="49"/>
+      <c r="B9" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="C9" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="D9" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="E9" s="1" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" ht="42" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="F9" s="1" t="s">
         <v>198</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="G9" s="1" t="s">
         <v>199</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="H9" s="1" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="42" customHeight="1">
+      <c r="A10" s="49"/>
+      <c r="B10" s="10" t="s">
         <v>200</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>201</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="D10" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="E10" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="F10" s="1" t="s">
         <v>204</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="G10" s="1" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" ht="42" customHeight="1">
-      <c r="A7" s="33"/>
-      <c r="B7" s="7" t="s">
+      <c r="H10" s="1" t="s">
         <v>206</v>
       </c>
-      <c r="C7" s="7" t="s">
+    </row>
+    <row r="11" spans="1:8" ht="34" customHeight="1">
+      <c r="A11" s="50" t="s">
         <v>207</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="B11" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="C11" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G7" s="1" t="s">
+      <c r="E11" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="F11" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="G11" s="9" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A8" s="34" t="s">
+      <c r="H11" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="B8" s="11" t="s">
+    </row>
+    <row r="12" spans="1:8" ht="42" customHeight="1">
+      <c r="A12" s="51"/>
+      <c r="B12" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="C12" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="D12" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="E12" s="1" t="s">
         <v>216</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="F12" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H12" s="1" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A9" s="35"/>
-      <c r="B9" s="10" t="s">
+    <row r="13" spans="1:8" ht="34" customHeight="1">
+      <c r="A13" s="43" t="s">
         <v>219</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="B13" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="C13" s="15" t="s">
         <v>221</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="D13" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="E13" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="H13" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="G9" s="1" t="s">
+    </row>
+    <row r="14" spans="1:8" ht="42" customHeight="1">
+      <c r="A14" s="44"/>
+      <c r="B14" s="14" t="s">
         <v>224</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="42" customHeight="1">
-      <c r="A10" s="35"/>
-      <c r="B10" s="10" t="s">
+      <c r="C14" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="D14" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E14" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F14" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="G14" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="G10" s="1" t="s">
+    </row>
+    <row r="15" spans="1:8" ht="34" customHeight="1">
+      <c r="A15" s="17" t="s">
         <v>230</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A11" s="36" t="s">
-        <v>232</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>233</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="H11" s="9" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" ht="42" customHeight="1">
-      <c r="A12" s="37"/>
-      <c r="B12" s="12" t="s">
-        <v>238</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>239</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>242</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A13" s="38" t="s">
-        <v>244</v>
-      </c>
-      <c r="B13" s="15" t="s">
-        <v>245</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>246</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>247</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="G13" s="9" t="s">
-        <v>246</v>
-      </c>
-      <c r="H13" s="9" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="42" customHeight="1">
-      <c r="A14" s="39"/>
-      <c r="B14" s="14" t="s">
-        <v>249</v>
-      </c>
-      <c r="C14" s="14" t="s">
-        <v>250</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>251</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A15" s="17" t="s">
-        <v>255</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>232</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="34" customHeight="1">
+      <c r="A16" s="58" t="s">
+        <v>237</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>238</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>233</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G16" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="42" customHeight="1">
+      <c r="A17" s="59"/>
+      <c r="B17" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="C17" s="18" t="s">
+        <v>241</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="34" customHeight="1">
+      <c r="A18" s="60" t="s">
+        <v>246</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>247</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="G18" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="34" customHeight="1">
+      <c r="A19" s="61"/>
+      <c r="B19" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="G19" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="D15" s="9" t="s">
+      <c r="H19" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="E15" s="9" t="s">
+    </row>
+    <row r="20" spans="1:8" ht="42" customHeight="1">
+      <c r="A20" s="46" t="s">
         <v>258</v>
       </c>
-      <c r="F15" s="9" t="s">
+      <c r="B20" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>259</v>
       </c>
-      <c r="G15" s="9" t="s">
+      <c r="D20" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="E20" s="9" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A16" s="42" t="s">
+      <c r="F20" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="B16" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="19" t="s">
+      <c r="G20" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H20" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="D16" s="9" t="s">
+    </row>
+    <row r="21" spans="1:8" ht="34" customHeight="1">
+      <c r="A21" s="47"/>
+      <c r="B21" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="E16" s="9" t="s">
-        <v>258</v>
-      </c>
-      <c r="F16" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="G16" s="9" t="s">
+      <c r="C21" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="H16" s="9" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="42" customHeight="1">
-      <c r="A17" s="43"/>
-      <c r="B17" s="18" t="s">
+      <c r="D21" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="C17" s="18" t="s">
-        <v>266</v>
-      </c>
-      <c r="D17" s="1" t="s">
+      <c r="E21" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="G17" s="1" t="s">
+      <c r="G21" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>270</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A18" s="44" t="s">
+    <row r="22" spans="1:8" ht="42" customHeight="1">
+      <c r="A22" s="47"/>
+      <c r="B22" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="B18" s="21" t="s">
+      <c r="C22" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="C18" s="21" t="s">
+      <c r="D22" s="1" t="s">
         <v>273</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E22" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="F22" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="F18" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="G18" s="9" t="s">
+      <c r="G22" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>276</v>
       </c>
-      <c r="H18" s="9" t="s">
+    </row>
+    <row r="23" spans="1:8" ht="34" customHeight="1">
+      <c r="A23" s="48" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A19" s="45"/>
-      <c r="B19" s="20" t="s">
+      <c r="B23" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>278</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="D23" s="9" t="s">
         <v>279</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="E23" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="E19" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="G19" s="1" t="s">
+      <c r="F23" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="G23" s="9" t="s">
         <v>282</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" ht="42" customHeight="1">
-      <c r="A20" s="32" t="s">
+      <c r="H23" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="C20" s="8" t="s">
+    </row>
+    <row r="24" spans="1:8" ht="42" customHeight="1">
+      <c r="A24" s="49"/>
+      <c r="B24" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="C24" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="D20" s="9" t="s">
+      <c r="D24" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="E20" s="9" t="s">
+      <c r="E24" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="F20" s="9" t="s">
+      <c r="F24" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="G20" s="9" t="s">
-        <v>122</v>
-      </c>
-      <c r="H20" s="9" t="s">
+      <c r="G24" s="1" t="s">
         <v>288</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A21" s="33"/>
-      <c r="B21" s="7" t="s">
+      <c r="H24" s="1" t="s">
         <v>289</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>290</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>293</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="42" customHeight="1">
-      <c r="A22" s="33"/>
-      <c r="B22" s="7" t="s">
-        <v>296</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>297</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>300</v>
-      </c>
-      <c r="G22" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="H22" s="1" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="33.950000000000003" customHeight="1">
-      <c r="A23" s="34" t="s">
-        <v>302</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="C23" s="11" t="s">
-        <v>303</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>305</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>306</v>
-      </c>
-      <c r="G23" s="9" t="s">
-        <v>307</v>
-      </c>
-      <c r="H23" s="9" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="42" customHeight="1">
-      <c r="A24" s="35"/>
-      <c r="B24" s="10" t="s">
-        <v>156</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>309</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>312</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>313</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="42" customHeight="1">
       <c r="A25" s="13" t="s">
-        <v>315</v>
+        <v>290</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>316</v>
+        <v>291</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>317</v>
+        <v>292</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>318</v>
+        <v>293</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>319</v>
+        <v>294</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>320</v>
+        <v>295</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>321</v>
+        <v>296</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>322</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="42" customHeight="1">
       <c r="A26" s="15" t="s">
-        <v>323</v>
+        <v>298</v>
       </c>
       <c r="B26" s="15" t="s">
-        <v>324</v>
+        <v>299</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>325</v>
+        <v>300</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>326</v>
+        <v>301</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>327</v>
+        <v>302</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>328</v>
+        <v>303</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>329</v>
+        <v>304</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>330</v>
+        <v>305</v>
       </c>
     </row>
   </sheetData>
@@ -4094,7 +4097,7 @@
     <tabColor rgb="FFB58B37"/>
   </sheetPr>
   <dimension ref="A1:G24"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="23" customWidth="1"/>
@@ -4105,7 +4108,7 @@
     <col min="7" max="7" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16.5">
+    <row r="1" spans="1:7" ht="17">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4115,17 +4118,17 @@
       <c r="G1" s="1"/>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1">
-      <c r="A2" s="29" t="s">
-        <v>331</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-    </row>
-    <row r="3" spans="1:7" ht="16.5">
+      <c r="A2" s="57" t="s">
+        <v>306</v>
+      </c>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+    </row>
+    <row r="3" spans="1:7" ht="17">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4134,7 +4137,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="16.5">
+    <row r="4" spans="1:7" ht="17">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -4145,391 +4148,391 @@
     </row>
     <row r="5" spans="1:7" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="42" customHeight="1">
+      <c r="A6" s="46" t="s">
+        <v>314</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>316</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>317</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>318</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>319</v>
+      </c>
+      <c r="G6" s="27"/>
+    </row>
+    <row r="7" spans="1:7" ht="42" customHeight="1">
+      <c r="A7" s="47"/>
+      <c r="B7" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>320</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="G7" s="28"/>
+    </row>
+    <row r="8" spans="1:7" ht="34" customHeight="1">
+      <c r="A8" s="47"/>
+      <c r="B8" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="G8" s="28"/>
+    </row>
+    <row r="9" spans="1:7" ht="42" customHeight="1">
+      <c r="A9" s="47"/>
+      <c r="B9" s="7" t="s">
+        <v>328</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>332</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="G9" s="28"/>
+    </row>
+    <row r="10" spans="1:7" ht="42" customHeight="1">
+      <c r="A10" s="47"/>
+      <c r="B10" s="7" t="s">
         <v>333</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C10" s="7" t="s">
         <v>334</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D10" s="1" t="s">
         <v>335</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E10" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F10" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G10" s="28"/>
+    </row>
+    <row r="11" spans="1:7" ht="42" customHeight="1">
+      <c r="A11" s="47"/>
+      <c r="B11" s="7" t="s">
         <v>338</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="42" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="C11" s="7" t="s">
         <v>339</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="D11" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="E11" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="G11" s="28"/>
+    </row>
+    <row r="12" spans="1:7" ht="42" customHeight="1">
+      <c r="A12" s="47"/>
+      <c r="B12" s="7" t="s">
         <v>342</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="C12" s="7" t="s">
         <v>343</v>
       </c>
-      <c r="F6" s="9" t="s">
+      <c r="D12" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="G6" s="27"/>
-    </row>
-    <row r="7" spans="1:7" ht="42" customHeight="1">
-      <c r="A7" s="33"/>
-      <c r="B7" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="C7" s="7" t="s">
+      <c r="E12" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="G12" s="28"/>
+    </row>
+    <row r="13" spans="1:7" ht="34" customHeight="1">
+      <c r="A13" s="48" t="s">
         <v>347</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="B13" s="11" t="s">
         <v>348</v>
       </c>
-      <c r="G7" s="28"/>
-    </row>
-    <row r="8" spans="1:7" ht="33.950000000000003" customHeight="1">
-      <c r="A8" s="33"/>
-      <c r="B8" s="7" t="s">
+      <c r="C13" s="11" t="s">
         <v>349</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D13" s="9" t="s">
         <v>350</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="E13" s="9" t="s">
         <v>351</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="F8" s="1" t="s">
+      <c r="F13" s="9" t="s">
         <v>352</v>
       </c>
-      <c r="G8" s="28"/>
-    </row>
-    <row r="9" spans="1:7" ht="42" customHeight="1">
-      <c r="A9" s="33"/>
-      <c r="B9" s="7" t="s">
+      <c r="G13" s="27"/>
+    </row>
+    <row r="14" spans="1:7" ht="34" customHeight="1">
+      <c r="A14" s="49"/>
+      <c r="B14" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="C14" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D14" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E14" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F14" s="1" t="s">
         <v>356</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="G14" s="28"/>
+    </row>
+    <row r="15" spans="1:7" ht="42" customHeight="1">
+      <c r="A15" s="49"/>
+      <c r="B15" s="10" t="s">
         <v>357</v>
       </c>
-      <c r="G9" s="28"/>
-    </row>
-    <row r="10" spans="1:7" ht="42" customHeight="1">
-      <c r="A10" s="33"/>
-      <c r="B10" s="7" t="s">
+      <c r="C15" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D15" s="1" t="s">
         <v>359</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="E15" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>360</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="G15" s="28"/>
+    </row>
+    <row r="16" spans="1:7" ht="42" customHeight="1">
+      <c r="A16" s="49"/>
+      <c r="B16" s="10" t="s">
         <v>361</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="C16" s="10" t="s">
         <v>362</v>
       </c>
-      <c r="G10" s="28"/>
-    </row>
-    <row r="11" spans="1:7" ht="42" customHeight="1">
-      <c r="A11" s="33"/>
-      <c r="B11" s="7" t="s">
+      <c r="D16" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="E16" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F16" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="G16" s="28"/>
+    </row>
+    <row r="17" spans="1:7" ht="42" customHeight="1">
+      <c r="A17" s="50" t="s">
         <v>365</v>
       </c>
-      <c r="E11" s="1" t="s">
-        <v>361</v>
-      </c>
-      <c r="F11" s="1" t="s">
+      <c r="B17" s="13" t="s">
         <v>366</v>
       </c>
-      <c r="G11" s="28"/>
-    </row>
-    <row r="12" spans="1:7" ht="42" customHeight="1">
-      <c r="A12" s="33"/>
-      <c r="B12" s="7" t="s">
+      <c r="C17" s="13" t="s">
         <v>367</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D17" s="9" t="s">
         <v>368</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="E17" s="9" t="s">
         <v>369</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F17" s="9" t="s">
         <v>370</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="G17" s="27"/>
+    </row>
+    <row r="18" spans="1:7" ht="42" customHeight="1">
+      <c r="A18" s="51"/>
+      <c r="B18" s="12" t="s">
         <v>371</v>
       </c>
-      <c r="G12" s="28"/>
-    </row>
-    <row r="13" spans="1:7" ht="33.950000000000003" customHeight="1">
-      <c r="A13" s="34" t="s">
+      <c r="C18" s="12" t="s">
         <v>372</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="D18" s="1" t="s">
         <v>373</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="E18" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="F18" s="1" t="s">
         <v>375</v>
       </c>
-      <c r="E13" s="9" t="s">
+      <c r="G18" s="28"/>
+    </row>
+    <row r="19" spans="1:7" ht="34" customHeight="1">
+      <c r="A19" s="51"/>
+      <c r="B19" s="12" t="s">
         <v>376</v>
       </c>
-      <c r="F13" s="9" t="s">
+      <c r="C19" s="12" t="s">
         <v>377</v>
       </c>
-      <c r="G13" s="27"/>
-    </row>
-    <row r="14" spans="1:7" ht="33.950000000000003" customHeight="1">
-      <c r="A14" s="35"/>
-      <c r="B14" s="10" t="s">
+      <c r="D19" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="E19" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F19" s="1" t="s">
         <v>379</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="G19" s="28"/>
+    </row>
+    <row r="20" spans="1:7" ht="34" customHeight="1">
+      <c r="A20" s="51"/>
+      <c r="B20" s="12" t="s">
         <v>380</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="C20" s="12" t="s">
         <v>381</v>
       </c>
-      <c r="G14" s="28"/>
-    </row>
-    <row r="15" spans="1:7" ht="42" customHeight="1">
-      <c r="A15" s="35"/>
-      <c r="B15" s="10" t="s">
+      <c r="D20" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="E20" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>383</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="G20" s="28"/>
+    </row>
+    <row r="21" spans="1:7" ht="42" customHeight="1">
+      <c r="A21" s="51"/>
+      <c r="B21" s="12" t="s">
         <v>384</v>
       </c>
-      <c r="E15" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="F15" s="1" t="s">
+      <c r="C21" s="12" t="s">
         <v>385</v>
       </c>
-      <c r="G15" s="28"/>
-    </row>
-    <row r="16" spans="1:7" ht="42" customHeight="1">
-      <c r="A16" s="35"/>
-      <c r="B16" s="10" t="s">
+      <c r="D21" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="E21" s="1" t="s">
         <v>387</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="F21" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="E16" s="1" t="s">
-        <v>376</v>
-      </c>
-      <c r="F16" s="1" t="s">
+      <c r="G21" s="28"/>
+    </row>
+    <row r="22" spans="1:7" ht="42" customHeight="1">
+      <c r="A22" s="51"/>
+      <c r="B22" s="12" t="s">
         <v>389</v>
       </c>
-      <c r="G16" s="28"/>
-    </row>
-    <row r="17" spans="1:7" ht="42" customHeight="1">
-      <c r="A17" s="36" t="s">
+      <c r="C22" s="12" t="s">
         <v>390</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="D22" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="E22" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="F22" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="G22" s="28"/>
+    </row>
+    <row r="23" spans="1:7" ht="42" customHeight="1">
+      <c r="A23" s="51"/>
+      <c r="B23" s="12" t="s">
         <v>393</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="C23" s="12" t="s">
         <v>394</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="D23" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="G17" s="27"/>
-    </row>
-    <row r="18" spans="1:7" ht="42" customHeight="1">
-      <c r="A18" s="37"/>
-      <c r="B18" s="12" t="s">
+      <c r="E23" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="F23" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="G23" s="28"/>
+    </row>
+    <row r="24" spans="1:7" ht="42" customHeight="1">
+      <c r="A24" s="51"/>
+      <c r="B24" s="12" t="s">
         <v>398</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="C24" s="12" t="s">
         <v>399</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="D24" s="1" t="s">
         <v>400</v>
-      </c>
-      <c r="G18" s="28"/>
-    </row>
-    <row r="19" spans="1:7" ht="33.950000000000003" customHeight="1">
-      <c r="A19" s="37"/>
-      <c r="B19" s="12" t="s">
-        <v>401</v>
-      </c>
-      <c r="C19" s="12" t="s">
-        <v>402</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="G19" s="28"/>
-    </row>
-    <row r="20" spans="1:7" ht="33.950000000000003" customHeight="1">
-      <c r="A20" s="37"/>
-      <c r="B20" s="12" t="s">
-        <v>405</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>406</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>407</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>408</v>
-      </c>
-      <c r="G20" s="28"/>
-    </row>
-    <row r="21" spans="1:7" ht="42" customHeight="1">
-      <c r="A21" s="37"/>
-      <c r="B21" s="12" t="s">
-        <v>409</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>410</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>413</v>
-      </c>
-      <c r="G21" s="28"/>
-    </row>
-    <row r="22" spans="1:7" ht="42" customHeight="1">
-      <c r="A22" s="37"/>
-      <c r="B22" s="12" t="s">
-        <v>414</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>415</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>209</v>
-      </c>
-      <c r="F22" s="1" t="s">
-        <v>417</v>
-      </c>
-      <c r="G22" s="28"/>
-    </row>
-    <row r="23" spans="1:7" ht="42" customHeight="1">
-      <c r="A23" s="37"/>
-      <c r="B23" s="12" t="s">
-        <v>418</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>419</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>420</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>421</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>422</v>
-      </c>
-      <c r="G23" s="28"/>
-    </row>
-    <row r="24" spans="1:7" ht="42" customHeight="1">
-      <c r="A24" s="37"/>
-      <c r="B24" s="12" t="s">
-        <v>423</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>424</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>425</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>5</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>426</v>
+        <v>401</v>
       </c>
       <c r="G24" s="28"/>
     </row>
@@ -4556,7 +4559,7 @@
     <tabColor rgb="FF8A737C"/>
   </sheetPr>
   <dimension ref="A1:F13"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="19" customWidth="1"/>
     <col min="2" max="2" width="27" customWidth="1"/>
@@ -4566,7 +4569,7 @@
     <col min="6" max="6" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.5">
+    <row r="1" spans="1:6" ht="17">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4575,16 +4578,16 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="29" t="s">
-        <v>427</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-    </row>
-    <row r="3" spans="1:6" ht="16.5">
+      <c r="A2" s="57" t="s">
+        <v>402</v>
+      </c>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+    </row>
+    <row r="3" spans="1:6" ht="17">
       <c r="A3" s="2"/>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -4592,7 +4595,7 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" spans="1:6" ht="16.5">
+    <row r="4" spans="1:6" ht="17">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -4602,153 +4605,153 @@
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1">
       <c r="A5" s="4" t="s">
-        <v>332</v>
+        <v>307</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>333</v>
+        <v>308</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>403</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="42" customHeight="1">
+      <c r="A6" s="46" t="s">
+        <v>405</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>407</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>409</v>
+      </c>
+      <c r="F6" s="27"/>
+    </row>
+    <row r="7" spans="1:6" ht="42" customHeight="1">
+      <c r="A7" s="47"/>
+      <c r="B7" s="7" t="s">
+        <v>410</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>411</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>413</v>
+      </c>
+      <c r="F7" s="28"/>
+    </row>
+    <row r="8" spans="1:6" ht="34" customHeight="1">
+      <c r="A8" s="48" t="s">
+        <v>414</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>418</v>
+      </c>
+      <c r="F8" s="27"/>
+    </row>
+    <row r="9" spans="1:6" ht="34" customHeight="1">
+      <c r="A9" s="49"/>
+      <c r="B9" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>422</v>
+      </c>
+      <c r="F9" s="28"/>
+    </row>
+    <row r="10" spans="1:6" ht="42" customHeight="1">
+      <c r="A10" s="49"/>
+      <c r="B10" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>424</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>425</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="F10" s="28"/>
+    </row>
+    <row r="11" spans="1:6" ht="34" customHeight="1">
+      <c r="A11" s="49"/>
+      <c r="B11" s="10" t="s">
+        <v>427</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>428</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="D11" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="F5" s="6" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="42" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="E11" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="F11" s="28"/>
+    </row>
+    <row r="12" spans="1:6" ht="42" customHeight="1">
+      <c r="A12" s="49"/>
+      <c r="B12" s="10" t="s">
         <v>431</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C12" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="D6" s="9" t="s">
+      <c r="D12" s="1" t="s">
         <v>433</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E12" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="F6" s="27"/>
-    </row>
-    <row r="7" spans="1:6" ht="42" customHeight="1">
-      <c r="A7" s="33"/>
-      <c r="B7" s="7" t="s">
+      <c r="F12" s="28"/>
+    </row>
+    <row r="13" spans="1:6" ht="34" customHeight="1">
+      <c r="A13" s="49"/>
+      <c r="B13" s="10" t="s">
         <v>435</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C13" s="10" t="s">
         <v>436</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>437</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>438</v>
-      </c>
-      <c r="F7" s="28"/>
-    </row>
-    <row r="8" spans="1:6" ht="33.950000000000003" customHeight="1">
-      <c r="A8" s="34" t="s">
-        <v>439</v>
-      </c>
-      <c r="B8" s="11" t="s">
-        <v>440</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>441</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>442</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>443</v>
-      </c>
-      <c r="F8" s="27"/>
-    </row>
-    <row r="9" spans="1:6" ht="33.950000000000003" customHeight="1">
-      <c r="A9" s="35"/>
-      <c r="B9" s="10" t="s">
-        <v>444</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>445</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>446</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>447</v>
-      </c>
-      <c r="F9" s="28"/>
-    </row>
-    <row r="10" spans="1:6" ht="42" customHeight="1">
-      <c r="A10" s="35"/>
-      <c r="B10" s="10" t="s">
-        <v>448</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>449</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>450</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>451</v>
-      </c>
-      <c r="F10" s="28"/>
-    </row>
-    <row r="11" spans="1:6" ht="33.950000000000003" customHeight="1">
-      <c r="A11" s="35"/>
-      <c r="B11" s="10" t="s">
-        <v>452</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>453</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>454</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>455</v>
-      </c>
-      <c r="F11" s="28"/>
-    </row>
-    <row r="12" spans="1:6" ht="42" customHeight="1">
-      <c r="A12" s="35"/>
-      <c r="B12" s="10" t="s">
-        <v>456</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>457</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>458</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>459</v>
-      </c>
-      <c r="F12" s="28"/>
-    </row>
-    <row r="13" spans="1:6" ht="33.950000000000003" customHeight="1">
-      <c r="A13" s="35"/>
-      <c r="B13" s="10" t="s">
-        <v>460</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>461</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>462</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>463</v>
       </c>
       <c r="F13" s="28"/>
     </row>
@@ -4765,5 +4768,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>